<commit_message>
se actualiza la salida de 'Datos_generales.xlsx', anexa las columnas de 'Laitutud' y 'Longitud'
</commit_message>
<xml_diff>
--- a/Datos_COTAINDOC.xlsx
+++ b/Datos_COTAINDOC.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,45 +444,55 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Latitud del Predio</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Longitud del Predio</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Puntaje_CULTURAL_PEDAGOGICO</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Puntaje_RIESGO_TERRITORIAL</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Puntaje_RIESGO_ESTRUCTURAL</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Puntaje_DEFICIT_COBERTURA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Puntaje_DEFICIT_CUALITATIVO</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Puntaje_INSTALACIONES_TECNICAS</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Puntaje_ACCESIBILIDAD</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Puntaje_CONFORT_AMBIENTAL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Puntaje_TOTAL</t>
         </is>
@@ -490,11 +500,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>219743000180</v>
+        <v>419743001118</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE RURAL MIXTO MIRAFLORES</t>
+          <t>CENTRO DOCENTE RURAL MIXTA CABUYAL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -509,44 +519,50 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMPIUILE</t>
+          <t>QUICHAYA</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>53.0441551724138</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>64.625</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
+        <v>42.40034965517242</v>
+      </c>
+      <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
-        <v>16.317</v>
-      </c>
       <c r="J2" t="n">
-        <v>29.4</v>
+        <v>23.7125</v>
       </c>
       <c r="K2" t="n">
-        <v>12.2375</v>
+        <v>82.917</v>
       </c>
       <c r="L2" t="n">
-        <v>46.39</v>
+        <v>64.2</v>
       </c>
       <c r="M2" t="n">
-        <v>16.3268</v>
+        <v>8.772499999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>29.79255689655172</v>
+        <v>16.66</v>
+      </c>
+      <c r="O2" t="n">
+        <v>66.3068</v>
+      </c>
+      <c r="P2" t="n">
+        <v>38.12114370689655</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>219743000953</v>
+        <v>219743000741</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ESCUELA ALTAMIRA QUICHAYA</t>
+          <t>I.E.T. AGROAMBIENTAL SEK BUVX FXIW LA GAITANA - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -565,40 +581,46 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>43.38364206896552</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>22.2</v>
+        <v>41.03319655172414</v>
       </c>
       <c r="I3" t="n">
-        <v>16.317</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>29.4</v>
+        <v>45.65000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>38.5</v>
+        <v>32.634</v>
       </c>
       <c r="L3" t="n">
-        <v>32.34</v>
+        <v>59</v>
       </c>
       <c r="M3" t="n">
-        <v>74.47019999999999</v>
+        <v>38.83000000000001</v>
       </c>
       <c r="N3" t="n">
-        <v>32.07635525862069</v>
+        <v>54.85999999999999</v>
+      </c>
+      <c r="O3" t="n">
+        <v>57.6436</v>
+      </c>
+      <c r="P3" t="n">
+        <v>41.20634956896551</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>419743001118</v>
+        <v>219743000953</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE RURAL MIXTA CABUYAL</t>
+          <t>ESCUELA ALTAMIRA QUICHAYA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -617,40 +639,46 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>42.40034965517242</v>
+        <v>2.7151502342512</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>-76.380505354855</v>
       </c>
       <c r="H4" t="n">
-        <v>23.7125</v>
+        <v>43.89452137931035</v>
       </c>
       <c r="I4" t="n">
-        <v>82.917</v>
+        <v>67.75</v>
       </c>
       <c r="J4" t="n">
-        <v>64.2</v>
+        <v>22.2</v>
       </c>
       <c r="K4" t="n">
-        <v>8.772499999999999</v>
+        <v>16.317</v>
       </c>
       <c r="L4" t="n">
-        <v>16.66</v>
+        <v>29.4</v>
       </c>
       <c r="M4" t="n">
-        <v>66.3068</v>
+        <v>38.5</v>
       </c>
       <c r="N4" t="n">
-        <v>38.12114370689655</v>
+        <v>56.77999999999999</v>
+      </c>
+      <c r="O4" t="n">
+        <v>57.81019999999999</v>
+      </c>
+      <c r="P4" t="n">
+        <v>41.58146517241379</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>219743000741</v>
+        <v>419743001151</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>I.E.T. AGROAMBIENTAL SEK BUVX FXIW LA GAITANA - SEDE PRINCIPAL</t>
+          <t>CENTRO DOCENTE BILING`E MARIPOSAS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -665,44 +693,50 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>QUICHAYA</t>
+          <t>PITAYO</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>40.96021379310345</v>
+        <v>2.7117753</v>
       </c>
       <c r="G5" t="n">
+        <v>-76.32434050000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>47.66512551724139</v>
+      </c>
+      <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
-        <v>45.65000000000001</v>
-      </c>
-      <c r="I5" t="n">
-        <v>32.634</v>
-      </c>
       <c r="J5" t="n">
-        <v>59</v>
+        <v>52.5</v>
       </c>
       <c r="K5" t="n">
-        <v>38.83000000000001</v>
+        <v>74.25900000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>50.41999999999999</v>
+        <v>44.2</v>
       </c>
       <c r="M5" t="n">
-        <v>57.6436</v>
+        <v>2.695</v>
       </c>
       <c r="N5" t="n">
-        <v>40.64222672413793</v>
+        <v>59.35999999999999</v>
+      </c>
+      <c r="O5" t="n">
+        <v>66.3068</v>
+      </c>
+      <c r="P5" t="n">
+        <v>43.37324068965518</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>419743001151</v>
+        <v>219743000031</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE BILING`E MARIPOSAS</t>
+          <t>CRISTO REY - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -717,44 +751,50 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PITAYO</t>
+          <t>TUMBURAO</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>47.66512551724139</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>52.5</v>
+        <v>58.54396413793104</v>
       </c>
       <c r="I6" t="n">
-        <v>74.25900000000001</v>
+        <v>80.5</v>
       </c>
       <c r="J6" t="n">
-        <v>44.2</v>
+        <v>14.7</v>
       </c>
       <c r="K6" t="n">
-        <v>2.695</v>
+        <v>16.317</v>
       </c>
       <c r="L6" t="n">
-        <v>59.35999999999999</v>
+        <v>39.6</v>
       </c>
       <c r="M6" t="n">
-        <v>66.3068</v>
+        <v>37.8675</v>
       </c>
       <c r="N6" t="n">
-        <v>43.37324068965518</v>
+        <v>51.31</v>
+      </c>
+      <c r="O6" t="n">
+        <v>61.642</v>
+      </c>
+      <c r="P6" t="n">
+        <v>45.06005801724137</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>219743000031</v>
+        <v>219743000180</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CRISTO REY - SEDE PRINCIPAL</t>
+          <t>CENTRO DOCENTE RURAL MIXTO MIRAFLORES</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -769,35 +809,41 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TUMBURAO</t>
+          <t>AMPIUILE</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>58.54396413793104</v>
+        <v>2.5539034007428</v>
       </c>
       <c r="G7" t="n">
-        <v>80.5</v>
+        <v>-76.425956006769</v>
       </c>
       <c r="H7" t="n">
-        <v>14.7</v>
+        <v>55.37960344827587</v>
       </c>
       <c r="I7" t="n">
+        <v>64.625</v>
+      </c>
+      <c r="J7" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="K7" t="n">
         <v>16.317</v>
       </c>
-      <c r="J7" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="K7" t="n">
-        <v>37.8675</v>
-      </c>
       <c r="L7" t="n">
-        <v>51.31</v>
+        <v>29.4</v>
       </c>
       <c r="M7" t="n">
-        <v>61.642</v>
+        <v>45.07250000000001</v>
       </c>
       <c r="N7" t="n">
-        <v>45.06005801724137</v>
+        <v>65.56999999999999</v>
+      </c>
+      <c r="O7" t="n">
+        <v>91.2968</v>
+      </c>
+      <c r="P7" t="n">
+        <v>48.73261293103449</v>
       </c>
     </row>
     <row r="8">
@@ -825,30 +871,36 @@
         </is>
       </c>
       <c r="F8" t="n">
+        <v>2.7769951593495</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-76.325073</v>
+      </c>
+      <c r="H8" t="n">
         <v>45.98875448275862</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>65.66499999999999</v>
       </c>
-      <c r="H8" t="n">
+      <c r="J8" t="n">
         <v>35.15</v>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>32.634</v>
       </c>
-      <c r="J8" t="n">
+      <c r="L8" t="n">
         <v>29.4</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>46.9975</v>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>66.56</v>
       </c>
-      <c r="M8" t="n">
+      <c r="O8" t="n">
         <v>69.97199999999999</v>
       </c>
-      <c r="N8" t="n">
+      <c r="P8" t="n">
         <v>49.04590681034483</v>
       </c>
     </row>
@@ -877,30 +929,36 @@
         </is>
       </c>
       <c r="F9" t="n">
+        <v>2.476093</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-76.39027900000001</v>
+      </c>
+      <c r="H9" t="n">
         <v>43.0658951724138</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>57.335</v>
       </c>
-      <c r="H9" t="n">
+      <c r="J9" t="n">
         <v>12.95</v>
       </c>
-      <c r="I9" t="n">
+      <c r="K9" t="n">
         <v>49.617</v>
       </c>
-      <c r="J9" t="n">
+      <c r="L9" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
         <v>38.88500000000001</v>
       </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
         <v>59.7362</v>
       </c>
-      <c r="M9" t="n">
+      <c r="O9" t="n">
         <v>70.4718</v>
       </c>
-      <c r="N9" t="n">
+      <c r="P9" t="n">
         <v>50.80761189655173</v>
       </c>
     </row>
@@ -929,30 +987,36 @@
         </is>
       </c>
       <c r="F10" t="n">
+        <v>2.498482</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-76.46150400000001</v>
+      </c>
+      <c r="H10" t="n">
         <v>47.10307241379311</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>24.5</v>
       </c>
-      <c r="H10" t="n">
+      <c r="J10" t="n">
         <v>50.375</v>
       </c>
-      <c r="I10" t="n">
+      <c r="K10" t="n">
         <v>74.25900000000001</v>
       </c>
-      <c r="J10" t="n">
+      <c r="L10" t="n">
         <v>71.90000000000001</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>46.2</v>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>76.56999999999999</v>
       </c>
-      <c r="M10" t="n">
+      <c r="O10" t="n">
         <v>16.3268</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>50.90423405172414</v>
       </c>
     </row>
@@ -981,30 +1045,36 @@
         </is>
       </c>
       <c r="F11" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-76.19</v>
+      </c>
+      <c r="H11" t="n">
         <v>43.64540689655173</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
         <v>66.15000000000001</v>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
         <v>65.934</v>
       </c>
-      <c r="J11" t="n">
+      <c r="L11" t="n">
         <v>64.2</v>
       </c>
-      <c r="K11" t="n">
+      <c r="M11" t="n">
         <v>38.17</v>
       </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
         <v>70.39</v>
       </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
         <v>65.807</v>
       </c>
-      <c r="N11" t="n">
+      <c r="P11" t="n">
         <v>51.78705086206897</v>
       </c>
     </row>
@@ -1033,30 +1103,36 @@
         </is>
       </c>
       <c r="F12" t="n">
+        <v>2.5467222</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-76.50475277777799</v>
+      </c>
+      <c r="H12" t="n">
         <v>69.61072620689654</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="n">
         <v>80.5</v>
       </c>
-      <c r="H12" t="n">
+      <c r="J12" t="n">
         <v>22.2</v>
       </c>
-      <c r="I12" t="n">
+      <c r="K12" t="n">
         <v>16.317</v>
       </c>
-      <c r="J12" t="n">
+      <c r="L12" t="n">
         <v>29.4</v>
       </c>
-      <c r="K12" t="n">
+      <c r="M12" t="n">
         <v>51.04000000000001</v>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>75.84</v>
       </c>
-      <c r="M12" t="n">
+      <c r="O12" t="n">
         <v>82.8002</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>53.46349077586207</v>
       </c>
     </row>
@@ -1085,30 +1161,36 @@
         </is>
       </c>
       <c r="F13" t="n">
+        <v>2.714233</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-76.439331</v>
+      </c>
+      <c r="H13" t="n">
         <v>73.31727724137932</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>61.5</v>
       </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
         <v>36.22499999999999</v>
       </c>
-      <c r="I13" t="n">
+      <c r="K13" t="n">
         <v>32.634</v>
       </c>
-      <c r="J13" t="n">
+      <c r="L13" t="n">
         <v>29.4</v>
       </c>
-      <c r="K13" t="n">
+      <c r="M13" t="n">
         <v>48.95</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>58.68999999999999</v>
       </c>
-      <c r="M13" t="n">
+      <c r="O13" t="n">
         <v>91.46339999999999</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>54.02245965517241</v>
       </c>
     </row>
@@ -1137,30 +1219,36 @@
         </is>
       </c>
       <c r="F14" t="n">
+        <v>2.482459</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-76.27980700000001</v>
+      </c>
+      <c r="H14" t="n">
         <v>43.23721862068966</v>
       </c>
-      <c r="G14" t="n">
+      <c r="I14" t="n">
         <v>55.25</v>
       </c>
-      <c r="H14" t="n">
+      <c r="J14" t="n">
         <v>47.22499999999999</v>
       </c>
-      <c r="I14" t="n">
+      <c r="K14" t="n">
         <v>71.81811000000002</v>
       </c>
-      <c r="J14" t="n">
+      <c r="L14" t="n">
         <v>54</v>
       </c>
-      <c r="K14" t="n">
+      <c r="M14" t="n">
         <v>19.14</v>
       </c>
-      <c r="L14" t="n">
+      <c r="N14" t="n">
         <v>66.88</v>
       </c>
-      <c r="M14" t="n">
+      <c r="O14" t="n">
         <v>82.96679999999999</v>
       </c>
-      <c r="N14" t="n">
+      <c r="P14" t="n">
         <v>55.06464107758621</v>
       </c>
     </row>
@@ -1189,30 +1277,36 @@
         </is>
       </c>
       <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>67.17647931034483</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>30.75</v>
       </c>
-      <c r="H15" t="n">
+      <c r="J15" t="n">
         <v>72.95</v>
       </c>
-      <c r="I15" t="n">
+      <c r="K15" t="n">
         <v>32.634</v>
       </c>
-      <c r="J15" t="n">
+      <c r="L15" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K15" t="n">
+      <c r="M15" t="n">
         <v>10.285</v>
       </c>
-      <c r="L15" t="n">
+      <c r="N15" t="n">
         <v>66.84</v>
       </c>
-      <c r="M15" t="n">
+      <c r="O15" t="n">
         <v>95.6284</v>
       </c>
-      <c r="N15" t="n">
+      <c r="P15" t="n">
         <v>56.3329849137931</v>
       </c>
     </row>
@@ -1241,30 +1335,36 @@
         </is>
       </c>
       <c r="F16" t="n">
+        <v>2.6109506</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-76.379982</v>
+      </c>
+      <c r="H16" t="n">
         <v>58.65146344827586</v>
       </c>
-      <c r="G16" t="n">
+      <c r="I16" t="n">
         <v>67.75</v>
       </c>
-      <c r="H16" t="n">
+      <c r="J16" t="n">
         <v>43.72499999999999</v>
       </c>
-      <c r="I16" t="n">
+      <c r="K16" t="n">
         <v>32.634</v>
       </c>
-      <c r="J16" t="n">
+      <c r="L16" t="n">
         <v>54.40000000000001</v>
       </c>
-      <c r="K16" t="n">
+      <c r="M16" t="n">
         <v>48.895</v>
       </c>
-      <c r="L16" t="n">
+      <c r="N16" t="n">
         <v>65.25</v>
       </c>
-      <c r="M16" t="n">
+      <c r="O16" t="n">
         <v>87.1318</v>
       </c>
-      <c r="N16" t="n">
+      <c r="P16" t="n">
         <v>57.30465793103448</v>
       </c>
     </row>
@@ -1293,30 +1393,36 @@
         </is>
       </c>
       <c r="F17" t="n">
+        <v>6.2529</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-75.5646</v>
+      </c>
+      <c r="H17" t="n">
         <v>63.81801310344828</v>
       </c>
-      <c r="G17" t="n">
+      <c r="I17" t="n">
         <v>0</v>
       </c>
-      <c r="H17" t="n">
+      <c r="J17" t="n">
         <v>76.09999999999999</v>
       </c>
-      <c r="I17" t="n">
+      <c r="K17" t="n">
         <v>95.571</v>
       </c>
-      <c r="J17" t="n">
+      <c r="L17" t="n">
         <v>64.2</v>
       </c>
-      <c r="K17" t="n">
+      <c r="M17" t="n">
         <v>40.975</v>
       </c>
-      <c r="L17" t="n">
+      <c r="N17" t="n">
         <v>48.41999999999999</v>
       </c>
-      <c r="M17" t="n">
+      <c r="O17" t="n">
         <v>70.1386</v>
       </c>
-      <c r="N17" t="n">
+      <c r="P17" t="n">
         <v>57.40282663793104</v>
       </c>
     </row>
@@ -1345,30 +1451,36 @@
         </is>
       </c>
       <c r="F18" t="n">
+        <v>2.657057</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-76.397313</v>
+      </c>
+      <c r="H18" t="n">
         <v>46.85212620689656</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>61.5</v>
       </c>
-      <c r="H18" t="n">
+      <c r="J18" t="n">
         <v>54.22500000000001</v>
       </c>
-      <c r="I18" t="n">
+      <c r="K18" t="n">
         <v>57.94200000000001</v>
       </c>
-      <c r="J18" t="n">
+      <c r="L18" t="n">
         <v>59</v>
       </c>
-      <c r="K18" t="n">
+      <c r="M18" t="n">
         <v>44.825</v>
       </c>
-      <c r="L18" t="n">
+      <c r="N18" t="n">
         <v>70.035</v>
       </c>
-      <c r="M18" t="n">
+      <c r="O18" t="n">
         <v>65.807</v>
       </c>
-      <c r="N18" t="n">
+      <c r="P18" t="n">
         <v>57.52326577586207</v>
       </c>
     </row>
@@ -1397,30 +1509,36 @@
         </is>
       </c>
       <c r="F19" t="n">
+        <v>2.7275498</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-76.3177017</v>
+      </c>
+      <c r="H19" t="n">
         <v>44.3922924137931</v>
       </c>
-      <c r="G19" t="n">
+      <c r="I19" t="n">
         <v>37</v>
       </c>
-      <c r="H19" t="n">
+      <c r="J19" t="n">
         <v>52.65000000000001</v>
       </c>
-      <c r="I19" t="n">
+      <c r="K19" t="n">
         <v>66.60000000000001</v>
       </c>
-      <c r="J19" t="n">
+      <c r="L19" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K19" t="n">
+      <c r="M19" t="n">
         <v>53.90000000000001</v>
       </c>
-      <c r="L19" t="n">
+      <c r="N19" t="n">
         <v>74.95</v>
       </c>
-      <c r="M19" t="n">
+      <c r="O19" t="n">
         <v>57.6436</v>
       </c>
-      <c r="N19" t="n">
+      <c r="P19" t="n">
         <v>57.69198655172413</v>
       </c>
     </row>
@@ -1449,30 +1567,36 @@
         </is>
       </c>
       <c r="F20" t="n">
+        <v>2.7591667</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-76.322777777778</v>
+      </c>
+      <c r="H20" t="n">
         <v>50.81792344827587</v>
       </c>
-      <c r="G20" t="n">
+      <c r="I20" t="n">
         <v>37</v>
       </c>
-      <c r="H20" t="n">
+      <c r="J20" t="n">
         <v>48.09999999999999</v>
       </c>
-      <c r="I20" t="n">
+      <c r="K20" t="n">
         <v>65.934</v>
       </c>
-      <c r="J20" t="n">
+      <c r="L20" t="n">
         <v>69.40000000000001</v>
       </c>
-      <c r="K20" t="n">
+      <c r="M20" t="n">
         <v>55.22000000000001</v>
       </c>
-      <c r="L20" t="n">
+      <c r="N20" t="n">
         <v>65.15000000000001</v>
       </c>
-      <c r="M20" t="n">
+      <c r="O20" t="n">
         <v>70.1386</v>
       </c>
-      <c r="N20" t="n">
+      <c r="P20" t="n">
         <v>57.72006543103448</v>
       </c>
     </row>
@@ -1501,30 +1625,36 @@
         </is>
       </c>
       <c r="F21" t="n">
+        <v>5.0599</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-75.48</v>
+      </c>
+      <c r="H21" t="n">
         <v>48.57497724137932</v>
       </c>
-      <c r="G21" t="n">
+      <c r="I21" t="n">
         <v>49</v>
       </c>
-      <c r="H21" t="n">
+      <c r="J21" t="n">
         <v>45.65000000000001</v>
       </c>
-      <c r="I21" t="n">
+      <c r="K21" t="n">
         <v>82.917</v>
       </c>
-      <c r="J21" t="n">
+      <c r="L21" t="n">
         <v>59</v>
       </c>
-      <c r="K21" t="n">
+      <c r="M21" t="n">
         <v>42.735</v>
       </c>
-      <c r="L21" t="n">
+      <c r="N21" t="n">
         <v>62.13</v>
       </c>
-      <c r="M21" t="n">
+      <c r="O21" t="n">
         <v>74.47019999999999</v>
       </c>
-      <c r="N21" t="n">
+      <c r="P21" t="n">
         <v>58.05964715517241</v>
       </c>
     </row>
@@ -1553,30 +1683,36 @@
         </is>
       </c>
       <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
         <v>48.76816689655173</v>
       </c>
-      <c r="G22" t="n">
+      <c r="I22" t="n">
         <v>37</v>
       </c>
-      <c r="H22" t="n">
+      <c r="J22" t="n">
         <v>48.09999999999999</v>
       </c>
-      <c r="I22" t="n">
+      <c r="K22" t="n">
         <v>82.917</v>
       </c>
-      <c r="J22" t="n">
+      <c r="L22" t="n">
         <v>64.2</v>
       </c>
-      <c r="K22" t="n">
+      <c r="M22" t="n">
         <v>49.19750000000001</v>
       </c>
-      <c r="L22" t="n">
+      <c r="N22" t="n">
         <v>58.52</v>
       </c>
-      <c r="M22" t="n">
+      <c r="O22" t="n">
         <v>78.6352</v>
       </c>
-      <c r="N22" t="n">
+      <c r="P22" t="n">
         <v>58.41723336206896</v>
       </c>
     </row>
@@ -1605,30 +1741,36 @@
         </is>
       </c>
       <c r="F23" t="n">
+        <v>2.6109894</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-76.3799837</v>
+      </c>
+      <c r="H23" t="n">
         <v>64.55585448275863</v>
       </c>
-      <c r="G23" t="n">
+      <c r="I23" t="n">
         <v>80.75</v>
       </c>
-      <c r="H23" t="n">
+      <c r="J23" t="n">
         <v>45.65000000000001</v>
       </c>
-      <c r="I23" t="n">
+      <c r="K23" t="n">
         <v>32.634</v>
       </c>
-      <c r="J23" t="n">
+      <c r="L23" t="n">
         <v>64.2</v>
       </c>
-      <c r="K23" t="n">
+      <c r="M23" t="n">
         <v>51.755</v>
       </c>
-      <c r="L23" t="n">
+      <c r="N23" t="n">
         <v>59.24999999999999</v>
       </c>
-      <c r="M23" t="n">
+      <c r="O23" t="n">
         <v>70.1386</v>
       </c>
-      <c r="N23" t="n">
+      <c r="P23" t="n">
         <v>58.61668181034483</v>
       </c>
     </row>
@@ -1657,40 +1799,46 @@
         </is>
       </c>
       <c r="F24" t="n">
+        <v>2.6960388333333</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-76.33137883333301</v>
+      </c>
+      <c r="H24" t="n">
         <v>68.32760344827587</v>
       </c>
-      <c r="G24" t="n">
+      <c r="I24" t="n">
         <v>61.5</v>
       </c>
-      <c r="H24" t="n">
+      <c r="J24" t="n">
         <v>25.9</v>
       </c>
-      <c r="I24" t="n">
+      <c r="K24" t="n">
         <v>65.934</v>
       </c>
-      <c r="J24" t="n">
+      <c r="L24" t="n">
         <v>59</v>
       </c>
-      <c r="K24" t="n">
+      <c r="M24" t="n">
         <v>49.61</v>
       </c>
-      <c r="L24" t="n">
+      <c r="N24" t="n">
         <v>68.31</v>
       </c>
-      <c r="M24" t="n">
+      <c r="O24" t="n">
         <v>74.3036</v>
       </c>
-      <c r="N24" t="n">
+      <c r="P24" t="n">
         <v>59.11065043103449</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>219743000015</v>
+        <v>219824000559</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE RURAL MIXTO LA PENA - CHERO</t>
+          <t>CENTRO DOCENTE ALTO MORENO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1700,49 +1848,55 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SILVIA</t>
+          <t>TOTORO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AMPIUILE</t>
+          <t>POLINDARA</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>58.43388896551724</v>
+        <v>2.4904333</v>
       </c>
       <c r="G25" t="n">
-        <v>49</v>
+        <v>-76.46464330000001</v>
       </c>
       <c r="H25" t="n">
-        <v>51.52500000000001</v>
+        <v>42.78043241379311</v>
       </c>
       <c r="I25" t="n">
-        <v>65.934</v>
+        <v>61.5</v>
       </c>
       <c r="J25" t="n">
-        <v>54</v>
+        <v>45.65000000000001</v>
       </c>
       <c r="K25" t="n">
-        <v>36.0525</v>
+        <v>66.60000000000001</v>
       </c>
       <c r="L25" t="n">
-        <v>67.14</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="M25" t="n">
-        <v>91.29679999999999</v>
+        <v>46.31</v>
       </c>
       <c r="N25" t="n">
-        <v>59.17277362068965</v>
+        <v>57.88999999999999</v>
+      </c>
+      <c r="O25" t="n">
+        <v>87.1318</v>
+      </c>
+      <c r="P25" t="n">
+        <v>59.65777905172414</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>219824000559</v>
+        <v>219824000192</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE ALTO MORENO</t>
+          <t>CENTRO DOCENTE CAMPO ALEGRE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1757,44 +1911,50 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>POLINDARA</t>
+          <t>PANIQUITA</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>42.78043241379311</v>
+        <v>2.52841</v>
       </c>
       <c r="G26" t="n">
-        <v>61.5</v>
+        <v>-76.4683</v>
       </c>
       <c r="H26" t="n">
-        <v>45.65000000000001</v>
+        <v>42.32295931034483</v>
       </c>
       <c r="I26" t="n">
-        <v>66.60000000000001</v>
+        <v>50</v>
       </c>
       <c r="J26" t="n">
-        <v>69.40000000000001</v>
+        <v>63.15000000000001</v>
       </c>
       <c r="K26" t="n">
-        <v>46.31</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L26" t="n">
-        <v>57.88999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="M26" t="n">
-        <v>87.1318</v>
+        <v>19.69</v>
       </c>
       <c r="N26" t="n">
-        <v>59.65777905172414</v>
+        <v>50.45</v>
+      </c>
+      <c r="O26" t="n">
+        <v>91.46339999999999</v>
+      </c>
+      <c r="P26" t="n">
+        <v>60.1470449137931</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>219824000192</v>
+        <v>219743000988</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE CAMPO ALEGRE</t>
+          <t>CENTRO DOCENTE RURAL MIXTO LAS DANTAS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1804,49 +1964,55 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TOTORO</t>
+          <t>SILVIA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PANIQUITA</t>
+          <t>QUICHAYA</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>42.32295931034483</v>
+        <v>3.49</v>
       </c>
       <c r="G27" t="n">
-        <v>50</v>
+        <v>-76.53</v>
       </c>
       <c r="H27" t="n">
-        <v>63.15000000000001</v>
+        <v>48.41241172413793</v>
       </c>
       <c r="I27" t="n">
-        <v>99.90000000000001</v>
+        <v>61.75</v>
       </c>
       <c r="J27" t="n">
+        <v>45.65000000000001</v>
+      </c>
+      <c r="K27" t="n">
+        <v>49.617</v>
+      </c>
+      <c r="L27" t="n">
         <v>64.2</v>
       </c>
-      <c r="K27" t="n">
-        <v>19.69</v>
-      </c>
-      <c r="L27" t="n">
-        <v>50.45</v>
-      </c>
       <c r="M27" t="n">
-        <v>91.46339999999999</v>
+        <v>60.17</v>
       </c>
       <c r="N27" t="n">
-        <v>60.1470449137931</v>
+        <v>60.31999999999999</v>
+      </c>
+      <c r="O27" t="n">
+        <v>91.2968</v>
+      </c>
+      <c r="P27" t="n">
+        <v>60.17702646551724</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>219743000988</v>
+        <v>219743000015</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE RURAL MIXTO LAS DANTAS</t>
+          <t>CENTRO DOCENTE RURAL MIXTO LA PENA - CHERO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1861,35 +2027,41 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>QUICHAYA</t>
+          <t>AMPIUILE</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>48.41241172413793</v>
+        <v>2.579316</v>
       </c>
       <c r="G28" t="n">
-        <v>61.75</v>
+        <v>-76.40201500000001</v>
       </c>
       <c r="H28" t="n">
-        <v>45.65000000000001</v>
+        <v>58.50687172413793</v>
       </c>
       <c r="I28" t="n">
-        <v>49.617</v>
+        <v>49</v>
       </c>
       <c r="J28" t="n">
+        <v>51.52500000000001</v>
+      </c>
+      <c r="K28" t="n">
+        <v>65.934</v>
+      </c>
+      <c r="L28" t="n">
         <v>64.2</v>
       </c>
-      <c r="K28" t="n">
-        <v>60.17</v>
-      </c>
-      <c r="L28" t="n">
-        <v>60.31999999999999</v>
-      </c>
       <c r="M28" t="n">
-        <v>91.2968</v>
+        <v>36.0525</v>
       </c>
       <c r="N28" t="n">
-        <v>60.17702646551724</v>
+        <v>67.14</v>
+      </c>
+      <c r="O28" t="n">
+        <v>91.29679999999999</v>
+      </c>
+      <c r="P28" t="n">
+        <v>60.45689646551725</v>
       </c>
     </row>
     <row r="29">
@@ -1917,30 +2089,36 @@
         </is>
       </c>
       <c r="F29" t="n">
+        <v>2.733145</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-76.34953400000001</v>
+      </c>
+      <c r="H29" t="n">
         <v>63.58063310344829</v>
       </c>
-      <c r="G29" t="n">
+      <c r="I29" t="n">
         <v>55.25</v>
       </c>
-      <c r="H29" t="n">
+      <c r="J29" t="n">
         <v>69.10000000000001</v>
       </c>
-      <c r="I29" t="n">
+      <c r="K29" t="n">
         <v>65.934</v>
       </c>
-      <c r="J29" t="n">
+      <c r="L29" t="n">
         <v>54</v>
       </c>
-      <c r="K29" t="n">
+      <c r="M29" t="n">
         <v>18.315</v>
       </c>
-      <c r="L29" t="n">
+      <c r="N29" t="n">
         <v>75.39</v>
       </c>
-      <c r="M29" t="n">
+      <c r="O29" t="n">
         <v>82.8002</v>
       </c>
-      <c r="N29" t="n">
+      <c r="P29" t="n">
         <v>60.54622913793104</v>
       </c>
     </row>
@@ -1969,30 +2147,36 @@
         </is>
       </c>
       <c r="F30" t="n">
+        <v>2.7400704142108</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-76.446283930994</v>
+      </c>
+      <c r="H30" t="n">
         <v>47.90983241379311</v>
       </c>
-      <c r="G30" t="n">
+      <c r="I30" t="n">
         <v>80.75</v>
       </c>
-      <c r="H30" t="n">
+      <c r="J30" t="n">
         <v>43.72499999999999</v>
       </c>
-      <c r="I30" t="n">
+      <c r="K30" t="n">
         <v>65.934</v>
       </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>69.2</v>
       </c>
-      <c r="K30" t="n">
+      <c r="M30" t="n">
         <v>53.90000000000001</v>
       </c>
-      <c r="L30" t="n">
+      <c r="N30" t="n">
         <v>63.31</v>
       </c>
-      <c r="M30" t="n">
+      <c r="O30" t="n">
         <v>61.64199999999998</v>
       </c>
-      <c r="N30" t="n">
+      <c r="P30" t="n">
         <v>60.79635405172414</v>
       </c>
     </row>
@@ -2021,30 +2205,36 @@
         </is>
       </c>
       <c r="F31" t="n">
+        <v>2.5796136684583</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-76.548874499544</v>
+      </c>
+      <c r="H31" t="n">
         <v>60.89881724137931</v>
       </c>
-      <c r="G31" t="n">
+      <c r="I31" t="n">
         <v>87.25</v>
       </c>
-      <c r="H31" t="n">
+      <c r="J31" t="n">
         <v>48.09999999999999</v>
       </c>
-      <c r="I31" t="n">
+      <c r="K31" t="n">
         <v>53.77950000000001</v>
       </c>
-      <c r="J31" t="n">
+      <c r="L31" t="n">
         <v>61.60000000000001</v>
       </c>
-      <c r="K31" t="n">
+      <c r="M31" t="n">
         <v>44.1925</v>
       </c>
-      <c r="L31" t="n">
+      <c r="N31" t="n">
         <v>70.45</v>
       </c>
-      <c r="M31" t="n">
+      <c r="O31" t="n">
         <v>61.642</v>
       </c>
-      <c r="N31" t="n">
+      <c r="P31" t="n">
         <v>60.98910215517241</v>
       </c>
     </row>
@@ -2073,30 +2263,36 @@
         </is>
       </c>
       <c r="F32" t="n">
+        <v>2.583234</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-76.47116699999999</v>
+      </c>
+      <c r="H32" t="n">
         <v>47.55573724137931</v>
       </c>
-      <c r="G32" t="n">
+      <c r="I32" t="n">
         <v>68</v>
       </c>
-      <c r="H32" t="n">
+      <c r="J32" t="n">
         <v>60.9</v>
       </c>
-      <c r="I32" t="n">
+      <c r="K32" t="n">
         <v>57.276</v>
       </c>
-      <c r="J32" t="n">
+      <c r="L32" t="n">
         <v>69.2</v>
       </c>
-      <c r="K32" t="n">
+      <c r="M32" t="n">
         <v>50.38</v>
       </c>
-      <c r="L32" t="n">
+      <c r="N32" t="n">
         <v>65.95</v>
       </c>
-      <c r="M32" t="n">
+      <c r="O32" t="n">
         <v>69.97199999999999</v>
       </c>
-      <c r="N32" t="n">
+      <c r="P32" t="n">
         <v>61.15421715517241</v>
       </c>
     </row>
@@ -2125,30 +2321,36 @@
         </is>
       </c>
       <c r="F33" t="n">
+        <v>2.6109789</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-76.3799805</v>
+      </c>
+      <c r="H33" t="n">
         <v>47.62872</v>
       </c>
-      <c r="G33" t="n">
+      <c r="I33" t="n">
         <v>55.25</v>
       </c>
-      <c r="H33" t="n">
+      <c r="J33" t="n">
         <v>58.60000000000001</v>
       </c>
-      <c r="I33" t="n">
+      <c r="K33" t="n">
         <v>74.25900000000001</v>
       </c>
-      <c r="J33" t="n">
+      <c r="L33" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K33" t="n">
+      <c r="M33" t="n">
         <v>46.2</v>
       </c>
-      <c r="L33" t="n">
+      <c r="N33" t="n">
         <v>66.11499999999999</v>
       </c>
-      <c r="M33" t="n">
+      <c r="O33" t="n">
         <v>70.1386</v>
       </c>
-      <c r="N33" t="n">
+      <c r="P33" t="n">
         <v>61.57391500000001</v>
       </c>
     </row>
@@ -2177,30 +2379,36 @@
         </is>
       </c>
       <c r="F34" t="n">
+        <v>2.6245808</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-76.3915926</v>
+      </c>
+      <c r="H34" t="n">
         <v>65.82747172413794</v>
       </c>
-      <c r="G34" t="n">
+      <c r="I34" t="n">
         <v>24.5</v>
       </c>
-      <c r="H34" t="n">
+      <c r="J34" t="n">
         <v>48.09999999999999</v>
       </c>
-      <c r="I34" t="n">
+      <c r="K34" t="n">
         <v>82.917</v>
       </c>
-      <c r="J34" t="n">
+      <c r="L34" t="n">
         <v>64.2</v>
       </c>
-      <c r="K34" t="n">
+      <c r="M34" t="n">
         <v>43.34</v>
       </c>
-      <c r="L34" t="n">
+      <c r="N34" t="n">
         <v>80.91</v>
       </c>
-      <c r="M34" t="n">
+      <c r="O34" t="n">
         <v>82.80019999999999</v>
       </c>
-      <c r="N34" t="n">
+      <c r="P34" t="n">
         <v>61.57433396551724</v>
       </c>
     </row>
@@ -2229,30 +2437,36 @@
         </is>
       </c>
       <c r="F35" t="n">
+        <v>2.707174</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-76.312241</v>
+      </c>
+      <c r="H35" t="n">
         <v>45.40970068965517</v>
       </c>
-      <c r="G35" t="n">
+      <c r="I35" t="n">
         <v>61.5</v>
       </c>
-      <c r="H35" t="n">
+      <c r="J35" t="n">
         <v>48.09999999999999</v>
       </c>
-      <c r="I35" t="n">
+      <c r="K35" t="n">
         <v>97.01289</v>
       </c>
-      <c r="J35" t="n">
+      <c r="L35" t="n">
         <v>64.2</v>
       </c>
-      <c r="K35" t="n">
+      <c r="M35" t="n">
         <v>38.6925</v>
       </c>
-      <c r="L35" t="n">
+      <c r="N35" t="n">
         <v>67.81</v>
       </c>
-      <c r="M35" t="n">
+      <c r="O35" t="n">
         <v>69.97199999999999</v>
       </c>
-      <c r="N35" t="n">
+      <c r="P35" t="n">
         <v>61.5871363362069</v>
       </c>
     </row>
@@ -2281,30 +2495,36 @@
         </is>
       </c>
       <c r="F36" t="n">
+        <v>2.7125038272673</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-76.32416419546099</v>
+      </c>
+      <c r="H36" t="n">
         <v>45.35812620689656</v>
       </c>
-      <c r="G36" t="n">
+      <c r="I36" t="n">
         <v>61.5</v>
       </c>
-      <c r="H36" t="n">
+      <c r="J36" t="n">
         <v>48.09999999999999</v>
       </c>
-      <c r="I36" t="n">
+      <c r="K36" t="n">
         <v>94.12911000000001</v>
       </c>
-      <c r="J36" t="n">
+      <c r="L36" t="n">
         <v>64.2</v>
       </c>
-      <c r="K36" t="n">
+      <c r="M36" t="n">
         <v>48.2625</v>
       </c>
-      <c r="L36" t="n">
+      <c r="N36" t="n">
         <v>64.52</v>
       </c>
-      <c r="M36" t="n">
+      <c r="O36" t="n">
         <v>70.1386</v>
       </c>
-      <c r="N36" t="n">
+      <c r="P36" t="n">
         <v>62.02604202586207</v>
       </c>
     </row>
@@ -2333,30 +2553,36 @@
         </is>
       </c>
       <c r="F37" t="n">
+        <v>2.684378</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-76.308464</v>
+      </c>
+      <c r="H37" t="n">
         <v>46.01914965517242</v>
       </c>
-      <c r="G37" t="n">
+      <c r="I37" t="n">
         <v>87.25</v>
       </c>
-      <c r="H37" t="n">
+      <c r="J37" t="n">
         <v>53.45</v>
       </c>
-      <c r="I37" t="n">
+      <c r="K37" t="n">
         <v>32.634</v>
       </c>
-      <c r="J37" t="n">
+      <c r="L37" t="n">
         <v>64.2</v>
       </c>
-      <c r="K37" t="n">
+      <c r="M37" t="n">
         <v>46.5575</v>
       </c>
-      <c r="L37" t="n">
+      <c r="N37" t="n">
         <v>77.41</v>
       </c>
-      <c r="M37" t="n">
+      <c r="O37" t="n">
         <v>91.46339999999999</v>
       </c>
-      <c r="N37" t="n">
+      <c r="P37" t="n">
         <v>62.37300620689655</v>
       </c>
     </row>
@@ -2385,30 +2611,36 @@
         </is>
       </c>
       <c r="F38" t="n">
+        <v>2.6368641042411</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-76.367885590881</v>
+      </c>
+      <c r="H38" t="n">
         <v>47.40147172413793</v>
       </c>
-      <c r="G38" t="n">
+      <c r="I38" t="n">
         <v>67.75</v>
       </c>
-      <c r="H38" t="n">
+      <c r="J38" t="n">
         <v>64.47500000000001</v>
       </c>
-      <c r="I38" t="n">
+      <c r="K38" t="n">
         <v>82.917</v>
       </c>
-      <c r="J38" t="n">
+      <c r="L38" t="n">
         <v>69.2</v>
       </c>
-      <c r="K38" t="n">
+      <c r="M38" t="n">
         <v>48.2075</v>
       </c>
-      <c r="L38" t="n">
+      <c r="N38" t="n">
         <v>61.78999999999999</v>
       </c>
-      <c r="M38" t="n">
+      <c r="O38" t="n">
         <v>57.6436</v>
       </c>
-      <c r="N38" t="n">
+      <c r="P38" t="n">
         <v>62.42307146551724</v>
       </c>
     </row>
@@ -2437,30 +2669,36 @@
         </is>
       </c>
       <c r="F39" t="n">
+        <v>2.771207</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-76.604446</v>
+      </c>
+      <c r="H39" t="n">
         <v>51.1861</v>
       </c>
-      <c r="G39" t="n">
+      <c r="I39" t="n">
         <v>0</v>
       </c>
-      <c r="H39" t="n">
+      <c r="J39" t="n">
         <v>77.87975</v>
       </c>
-      <c r="I39" t="n">
+      <c r="K39" t="n">
         <v>95.61096000000001</v>
       </c>
-      <c r="J39" t="n">
+      <c r="L39" t="n">
         <v>63.55</v>
       </c>
-      <c r="K39" t="n">
+      <c r="M39" t="n">
         <v>64.24000000000001</v>
       </c>
-      <c r="L39" t="n">
+      <c r="N39" t="n">
         <v>72.27</v>
       </c>
-      <c r="M39" t="n">
+      <c r="O39" t="n">
         <v>78.6352</v>
       </c>
-      <c r="N39" t="n">
+      <c r="P39" t="n">
         <v>62.92150125</v>
       </c>
     </row>
@@ -2489,30 +2727,36 @@
         </is>
       </c>
       <c r="F40" t="n">
+        <v>6.2529</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-75.5646</v>
+      </c>
+      <c r="H40" t="n">
         <v>47.88613448275862</v>
       </c>
-      <c r="G40" t="n">
+      <c r="I40" t="n">
         <v>61.5</v>
       </c>
-      <c r="H40" t="n">
+      <c r="J40" t="n">
         <v>59.675</v>
       </c>
-      <c r="I40" t="n">
+      <c r="K40" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="J40" t="n">
+      <c r="L40" t="n">
         <v>64.2</v>
       </c>
-      <c r="K40" t="n">
+      <c r="M40" t="n">
         <v>43.395</v>
       </c>
-      <c r="L40" t="n">
+      <c r="N40" t="n">
         <v>63.31999999999999</v>
       </c>
-      <c r="M40" t="n">
+      <c r="O40" t="n">
         <v>70.1386</v>
       </c>
-      <c r="N40" t="n">
+      <c r="P40" t="n">
         <v>63.75184181034483</v>
       </c>
     </row>
@@ -2541,30 +2785,36 @@
         </is>
       </c>
       <c r="F41" t="n">
+        <v>6.2529</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-75.5646</v>
+      </c>
+      <c r="H41" t="n">
         <v>47.03008965517242</v>
       </c>
-      <c r="G41" t="n">
+      <c r="I41" t="n">
         <v>67.75</v>
       </c>
-      <c r="H41" t="n">
+      <c r="J41" t="n">
         <v>73.65000000000001</v>
       </c>
-      <c r="I41" t="n">
+      <c r="K41" t="n">
         <v>82.917</v>
       </c>
-      <c r="J41" t="n">
+      <c r="L41" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K41" t="n">
+      <c r="M41" t="n">
         <v>40.755</v>
       </c>
-      <c r="L41" t="n">
+      <c r="N41" t="n">
         <v>58.49999999999999</v>
       </c>
-      <c r="M41" t="n">
+      <c r="O41" t="n">
         <v>66.14019999999999</v>
       </c>
-      <c r="N41" t="n">
+      <c r="P41" t="n">
         <v>63.89278620689655</v>
       </c>
     </row>
@@ -2593,30 +2843,36 @@
         </is>
       </c>
       <c r="F42" t="n">
+        <v>2.611862999513</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-76.378959043397</v>
+      </c>
+      <c r="H42" t="n">
         <v>64.82528965517241</v>
       </c>
-      <c r="G42" t="n">
+      <c r="I42" t="n">
         <v>80.75</v>
       </c>
-      <c r="H42" t="n">
+      <c r="J42" t="n">
         <v>35.15</v>
       </c>
-      <c r="I42" t="n">
+      <c r="K42" t="n">
         <v>91.24200000000002</v>
       </c>
-      <c r="J42" t="n">
+      <c r="L42" t="n">
         <v>59</v>
       </c>
-      <c r="K42" t="n">
+      <c r="M42" t="n">
         <v>34.5125</v>
       </c>
-      <c r="L42" t="n">
+      <c r="N42" t="n">
         <v>66.27</v>
       </c>
-      <c r="M42" t="n">
+      <c r="O42" t="n">
         <v>87.1318</v>
       </c>
-      <c r="N42" t="n">
+      <c r="P42" t="n">
         <v>64.86019870689654</v>
       </c>
     </row>
@@ -2645,30 +2901,36 @@
         </is>
       </c>
       <c r="F43" t="n">
+        <v>2.443201</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-76.6044315</v>
+      </c>
+      <c r="H43" t="n">
         <v>63.11692068965517</v>
       </c>
-      <c r="G43" t="n">
+      <c r="I43" t="n">
         <v>82.91499999999999</v>
       </c>
-      <c r="H43" t="n">
+      <c r="J43" t="n">
         <v>70.61725</v>
       </c>
-      <c r="I43" t="n">
+      <c r="K43" t="n">
         <v>57.94200000000001</v>
       </c>
-      <c r="J43" t="n">
+      <c r="L43" t="n">
         <v>60.73400000000001</v>
       </c>
-      <c r="K43" t="n">
+      <c r="M43" t="n">
         <v>28.49</v>
       </c>
-      <c r="L43" t="n">
+      <c r="N43" t="n">
         <v>72.27</v>
       </c>
-      <c r="M43" t="n">
+      <c r="O43" t="n">
         <v>82.96679999999999</v>
       </c>
-      <c r="N43" t="n">
+      <c r="P43" t="n">
         <v>64.88149633620691</v>
       </c>
     </row>
@@ -2697,30 +2959,36 @@
         </is>
       </c>
       <c r="F44" t="n">
+        <v>2.533274</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-76.315173</v>
+      </c>
+      <c r="H44" t="n">
         <v>62.56064896551725</v>
       </c>
-      <c r="G44" t="n">
+      <c r="I44" t="n">
         <v>80.5</v>
       </c>
-      <c r="H44" t="n">
+      <c r="J44" t="n">
         <v>66.91250000000001</v>
       </c>
-      <c r="I44" t="n">
+      <c r="K44" t="n">
         <v>68.34825000000001</v>
       </c>
-      <c r="J44" t="n">
+      <c r="L44" t="n">
         <v>59</v>
       </c>
-      <c r="K44" t="n">
+      <c r="M44" t="n">
         <v>35.9975</v>
       </c>
-      <c r="L44" t="n">
+      <c r="N44" t="n">
         <v>62.95999999999999</v>
       </c>
-      <c r="M44" t="n">
+      <c r="O44" t="n">
         <v>82.96679999999999</v>
       </c>
-      <c r="N44" t="n">
+      <c r="P44" t="n">
         <v>64.90571237068966</v>
       </c>
     </row>
@@ -2749,30 +3017,36 @@
         </is>
       </c>
       <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
         <v>58.5736724137931</v>
       </c>
-      <c r="G45" t="n">
+      <c r="I45" t="n">
         <v>74.25</v>
       </c>
-      <c r="H45" t="n">
+      <c r="J45" t="n">
         <v>60.375</v>
       </c>
-      <c r="I45" t="n">
+      <c r="K45" t="n">
         <v>91.4085</v>
       </c>
-      <c r="J45" t="n">
+      <c r="L45" t="n">
         <v>77</v>
       </c>
-      <c r="K45" t="n">
+      <c r="M45" t="n">
         <v>36.65750000000001</v>
       </c>
-      <c r="L45" t="n">
+      <c r="N45" t="n">
         <v>59.88</v>
       </c>
-      <c r="M45" t="n">
+      <c r="O45" t="n">
         <v>65.80699999999999</v>
       </c>
-      <c r="N45" t="n">
+      <c r="P45" t="n">
         <v>65.49395905172415</v>
       </c>
     </row>
@@ -2801,31 +3075,37 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>53.39058</v>
+        <v>2.7175084988588</v>
       </c>
       <c r="G46" t="n">
+        <v>-76.382177458998</v>
+      </c>
+      <c r="H46" t="n">
+        <v>53.46356275862069</v>
+      </c>
+      <c r="I46" t="n">
         <v>88.38499999999999</v>
       </c>
-      <c r="H46" t="n">
+      <c r="J46" t="n">
         <v>55.90000000000001</v>
       </c>
-      <c r="I46" t="n">
+      <c r="K46" t="n">
         <v>65.934</v>
       </c>
-      <c r="J46" t="n">
+      <c r="L46" t="n">
         <v>64.30000000000001</v>
       </c>
-      <c r="K46" t="n">
+      <c r="M46" t="n">
         <v>45.54</v>
       </c>
-      <c r="L46" t="n">
+      <c r="N46" t="n">
         <v>82.13979999999999</v>
       </c>
-      <c r="M46" t="n">
+      <c r="O46" t="n">
         <v>69.97199999999999</v>
       </c>
-      <c r="N46" t="n">
-        <v>65.6951725</v>
+      <c r="P46" t="n">
+        <v>65.70429534482759</v>
       </c>
     </row>
     <row r="47">
@@ -2853,30 +3133,36 @@
         </is>
       </c>
       <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
         <v>80.75573724137932</v>
       </c>
-      <c r="G47" t="n">
+      <c r="I47" t="n">
         <v>67.75</v>
       </c>
-      <c r="H47" t="n">
+      <c r="J47" t="n">
         <v>55.90000000000001</v>
       </c>
-      <c r="I47" t="n">
+      <c r="K47" t="n">
         <v>65.934</v>
       </c>
-      <c r="J47" t="n">
+      <c r="L47" t="n">
         <v>59.2</v>
       </c>
-      <c r="K47" t="n">
+      <c r="M47" t="n">
         <v>45.595</v>
       </c>
-      <c r="L47" t="n">
+      <c r="N47" t="n">
         <v>66.81</v>
       </c>
-      <c r="M47" t="n">
+      <c r="O47" t="n">
         <v>87.1318</v>
       </c>
-      <c r="N47" t="n">
+      <c r="P47" t="n">
         <v>66.13456715517242</v>
       </c>
     </row>
@@ -2905,30 +3191,36 @@
         </is>
       </c>
       <c r="F48" t="n">
+        <v>2.734253</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-76.329956</v>
+      </c>
+      <c r="H48" t="n">
         <v>48.60514344827587</v>
       </c>
-      <c r="G48" t="n">
+      <c r="I48" t="n">
         <v>74.25</v>
       </c>
-      <c r="H48" t="n">
+      <c r="J48" t="n">
         <v>77.6155</v>
       </c>
-      <c r="I48" t="n">
+      <c r="K48" t="n">
         <v>96.43680000000001</v>
       </c>
-      <c r="J48" t="n">
+      <c r="L48" t="n">
         <v>70.87200000000001</v>
       </c>
-      <c r="K48" t="n">
+      <c r="M48" t="n">
         <v>48.3175</v>
       </c>
-      <c r="L48" t="n">
+      <c r="N48" t="n">
         <v>64.13</v>
       </c>
-      <c r="M48" t="n">
+      <c r="O48" t="n">
         <v>49.31359999999999</v>
       </c>
-      <c r="N48" t="n">
+      <c r="P48" t="n">
         <v>66.19256793103449</v>
       </c>
     </row>
@@ -2957,30 +3249,36 @@
         </is>
       </c>
       <c r="F49" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-75.59999999999999</v>
+      </c>
+      <c r="H49" t="n">
         <v>65.08539448275863</v>
       </c>
-      <c r="G49" t="n">
+      <c r="I49" t="n">
         <v>24.5</v>
       </c>
-      <c r="H49" t="n">
+      <c r="J49" t="n">
         <v>81.80000000000001</v>
       </c>
-      <c r="I49" t="n">
+      <c r="K49" t="n">
         <v>82.917</v>
       </c>
-      <c r="J49" t="n">
+      <c r="L49" t="n">
         <v>69.40000000000001</v>
       </c>
-      <c r="K49" t="n">
+      <c r="M49" t="n">
         <v>56.705</v>
       </c>
-      <c r="L49" t="n">
+      <c r="N49" t="n">
         <v>54.63999999999999</v>
       </c>
-      <c r="M49" t="n">
+      <c r="O49" t="n">
         <v>95.6284</v>
       </c>
-      <c r="N49" t="n">
+      <c r="P49" t="n">
         <v>66.33447431034483</v>
       </c>
     </row>
@@ -3009,30 +3307,36 @@
         </is>
       </c>
       <c r="F50" t="n">
+        <v>23.037529</v>
+      </c>
+      <c r="G50" t="n">
+        <v>113.846692</v>
+      </c>
+      <c r="H50" t="n">
         <v>62.49894275862069</v>
       </c>
-      <c r="G50" t="n">
+      <c r="I50" t="n">
         <v>80.5</v>
       </c>
-      <c r="H50" t="n">
+      <c r="J50" t="n">
         <v>80.91250000000001</v>
       </c>
-      <c r="I50" t="n">
+      <c r="K50" t="n">
         <v>58.10850000000001</v>
       </c>
-      <c r="J50" t="n">
+      <c r="L50" t="n">
         <v>61.60000000000001</v>
       </c>
-      <c r="K50" t="n">
+      <c r="M50" t="n">
         <v>41.41500000000001</v>
       </c>
-      <c r="L50" t="n">
+      <c r="N50" t="n">
         <v>64.675</v>
       </c>
-      <c r="M50" t="n">
+      <c r="O50" t="n">
         <v>82.8002</v>
       </c>
-      <c r="N50" t="n">
+      <c r="P50" t="n">
         <v>66.56376784482759</v>
       </c>
     </row>
@@ -3061,30 +3365,36 @@
         </is>
       </c>
       <c r="F51" t="n">
+        <v>2.520396</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-76.31965099999999</v>
+      </c>
+      <c r="H51" t="n">
         <v>41.79061448275862</v>
       </c>
-      <c r="G51" t="n">
+      <c r="I51" t="n">
         <v>63.585</v>
       </c>
-      <c r="H51" t="n">
+      <c r="J51" t="n">
         <v>64.575</v>
       </c>
-      <c r="I51" t="n">
+      <c r="K51" t="n">
         <v>91.88469000000001</v>
       </c>
-      <c r="J51" t="n">
+      <c r="L51" t="n">
         <v>65.24000000000001</v>
       </c>
-      <c r="K51" t="n">
+      <c r="M51" t="n">
         <v>48.29</v>
       </c>
-      <c r="L51" t="n">
+      <c r="N51" t="n">
         <v>70.78</v>
       </c>
-      <c r="M51" t="n">
+      <c r="O51" t="n">
         <v>87.1318</v>
       </c>
-      <c r="N51" t="n">
+      <c r="P51" t="n">
         <v>66.65963806034483</v>
       </c>
     </row>
@@ -3113,30 +3423,36 @@
         </is>
       </c>
       <c r="F52" t="n">
+        <v>2.610953</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-76.379982</v>
+      </c>
+      <c r="H52" t="n">
         <v>49.04304</v>
       </c>
-      <c r="G52" t="n">
+      <c r="I52" t="n">
         <v>80.75</v>
       </c>
-      <c r="H52" t="n">
+      <c r="J52" t="n">
         <v>69.10000000000001</v>
       </c>
-      <c r="I52" t="n">
+      <c r="K52" t="n">
         <v>91.24200000000002</v>
       </c>
-      <c r="J52" t="n">
+      <c r="L52" t="n">
         <v>69.40000000000001</v>
       </c>
-      <c r="K52" t="n">
+      <c r="M52" t="n">
         <v>41.6625</v>
       </c>
-      <c r="L52" t="n">
+      <c r="N52" t="n">
         <v>62.18999999999999</v>
       </c>
-      <c r="M52" t="n">
+      <c r="O52" t="n">
         <v>74.47019999999999</v>
       </c>
-      <c r="N52" t="n">
+      <c r="P52" t="n">
         <v>67.23221750000002</v>
       </c>
     </row>
@@ -3165,30 +3481,36 @@
         </is>
       </c>
       <c r="F53" t="n">
+        <v>2.7072664</v>
+      </c>
+      <c r="G53" t="n">
+        <v>-76.39857000000001</v>
+      </c>
+      <c r="H53" t="n">
         <v>44.84678896551724</v>
       </c>
-      <c r="G53" t="n">
+      <c r="I53" t="n">
         <v>78.58500000000001</v>
       </c>
-      <c r="H53" t="n">
+      <c r="J53" t="n">
         <v>61.05</v>
       </c>
-      <c r="I53" t="n">
+      <c r="K53" t="n">
         <v>82.917</v>
       </c>
-      <c r="J53" t="n">
+      <c r="L53" t="n">
         <v>71.80000000000001</v>
       </c>
-      <c r="K53" t="n">
+      <c r="M53" t="n">
         <v>48.62</v>
       </c>
-      <c r="L53" t="n">
+      <c r="N53" t="n">
         <v>71.3</v>
       </c>
-      <c r="M53" t="n">
+      <c r="O53" t="n">
         <v>87.1318</v>
       </c>
-      <c r="N53" t="n">
+      <c r="P53" t="n">
         <v>68.28132362068966</v>
       </c>
     </row>
@@ -3217,30 +3539,36 @@
         </is>
       </c>
       <c r="F54" t="n">
+        <v>2.486517</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-76.448014</v>
+      </c>
+      <c r="H54" t="n">
         <v>68.20258827586207</v>
       </c>
-      <c r="G54" t="n">
+      <c r="I54" t="n">
         <v>55.25</v>
       </c>
-      <c r="H54" t="n">
+      <c r="J54" t="n">
         <v>67.56224999999999</v>
       </c>
-      <c r="I54" t="n">
+      <c r="K54" t="n">
         <v>87.87204000000001</v>
       </c>
-      <c r="J54" t="n">
+      <c r="L54" t="n">
         <v>62.714</v>
       </c>
-      <c r="K54" t="n">
+      <c r="M54" t="n">
         <v>49.005</v>
       </c>
-      <c r="L54" t="n">
+      <c r="N54" t="n">
         <v>68.7</v>
       </c>
-      <c r="M54" t="n">
+      <c r="O54" t="n">
         <v>91.46339999999999</v>
       </c>
-      <c r="N54" t="n">
+      <c r="P54" t="n">
         <v>68.84615978448277</v>
       </c>
     </row>
@@ -3269,30 +3597,36 @@
         </is>
       </c>
       <c r="F55" t="n">
+        <v>2.740025</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-76.535487</v>
+      </c>
+      <c r="H55" t="n">
         <v>47.52093448275863</v>
       </c>
-      <c r="G55" t="n">
+      <c r="I55" t="n">
         <v>37</v>
       </c>
-      <c r="H55" t="n">
+      <c r="J55" t="n">
         <v>74.40774999999999</v>
       </c>
-      <c r="I55" t="n">
+      <c r="K55" t="n">
         <v>97.01289</v>
       </c>
-      <c r="J55" t="n">
+      <c r="L55" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K55" t="n">
+      <c r="M55" t="n">
         <v>55.1375</v>
       </c>
-      <c r="L55" t="n">
+      <c r="N55" t="n">
         <v>78.59</v>
       </c>
-      <c r="M55" t="n">
+      <c r="O55" t="n">
         <v>86.9652</v>
       </c>
-      <c r="N55" t="n">
+      <c r="P55" t="n">
         <v>68.87928431034483</v>
       </c>
     </row>
@@ -3321,40 +3655,46 @@
         </is>
       </c>
       <c r="F56" t="n">
+        <v>2.611422</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-76.379839</v>
+      </c>
+      <c r="H56" t="n">
         <v>59.27516551724138</v>
       </c>
-      <c r="G56" t="n">
+      <c r="I56" t="n">
         <v>80.75</v>
       </c>
-      <c r="H56" t="n">
+      <c r="J56" t="n">
         <v>65.60000000000001</v>
       </c>
-      <c r="I56" t="n">
+      <c r="K56" t="n">
         <v>82.75050000000002</v>
       </c>
-      <c r="J56" t="n">
+      <c r="L56" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K56" t="n">
+      <c r="M56" t="n">
         <v>53.2125</v>
       </c>
-      <c r="L56" t="n">
+      <c r="N56" t="n">
         <v>62.81999999999999</v>
       </c>
-      <c r="M56" t="n">
+      <c r="O56" t="n">
         <v>74.3036</v>
       </c>
-      <c r="N56" t="n">
+      <c r="P56" t="n">
         <v>69.13897068965517</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>219824000206</v>
+        <v>219548000825</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CENTRO DOCENTE RURAL MIXTA BUENAVISTA</t>
+          <t>ESCUELA RURAL MIXTA VALPARAISO</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3364,49 +3704,55 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>TOTORO</t>
+          <t>PIENDAMO</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>PANIQUITA</t>
+          <t>LA MARIA</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>64.48613448275862</v>
+        <v>2.7160033694779</v>
       </c>
       <c r="G57" t="n">
-        <v>24.5</v>
+        <v>-76.603611220213</v>
       </c>
       <c r="H57" t="n">
-        <v>81.19974999999999</v>
+        <v>64.79993172413793</v>
       </c>
       <c r="I57" t="n">
-        <v>66.24036000000001</v>
+        <v>61.5</v>
       </c>
       <c r="J57" t="n">
-        <v>79.166</v>
+        <v>79.5125</v>
       </c>
       <c r="K57" t="n">
-        <v>61.38</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L57" t="n">
-        <v>82.73</v>
+        <v>65.5</v>
       </c>
       <c r="M57" t="n">
-        <v>99.95999999999999</v>
+        <v>51.0125</v>
       </c>
       <c r="N57" t="n">
-        <v>69.95778056034483</v>
+        <v>70.51000000000001</v>
+      </c>
+      <c r="O57" t="n">
+        <v>70.4718</v>
+      </c>
+      <c r="P57" t="n">
+        <v>70.40084146551723</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>219548000825</v>
+        <v>219824000206</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ESCUELA RURAL MIXTA VALPARAISO</t>
+          <t>CENTRO DOCENTE RURAL MIXTA BUENAVISTA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3416,40 +3762,46 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>PIENDAMO</t>
+          <t>TOTORO</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>LA MARIA</t>
+          <t>PANIQUITA</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>64.79993172413793</v>
+        <v>2.6941972</v>
       </c>
       <c r="G58" t="n">
-        <v>61.5</v>
+        <v>-76.33258333333301</v>
       </c>
       <c r="H58" t="n">
-        <v>79.5125</v>
+        <v>64.63210000000001</v>
       </c>
       <c r="I58" t="n">
-        <v>99.90000000000001</v>
+        <v>24.5</v>
       </c>
       <c r="J58" t="n">
-        <v>65.5</v>
+        <v>81.19974999999999</v>
       </c>
       <c r="K58" t="n">
-        <v>51.0125</v>
+        <v>77.33925000000002</v>
       </c>
       <c r="L58" t="n">
-        <v>70.51000000000001</v>
+        <v>79.166</v>
       </c>
       <c r="M58" t="n">
-        <v>70.4718</v>
+        <v>61.38</v>
       </c>
       <c r="N58" t="n">
-        <v>70.40084146551723</v>
+        <v>82.73</v>
+      </c>
+      <c r="O58" t="n">
+        <v>99.95999999999999</v>
+      </c>
+      <c r="P58" t="n">
+        <v>71.3633875</v>
       </c>
     </row>
     <row r="59">
@@ -3477,30 +3829,36 @@
         </is>
       </c>
       <c r="F59" t="n">
+        <v>2.734253</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-76.329956</v>
+      </c>
+      <c r="H59" t="n">
         <v>65.5267827586207</v>
       </c>
-      <c r="G59" t="n">
+      <c r="I59" t="n">
         <v>80.5</v>
       </c>
-      <c r="H59" t="n">
+      <c r="J59" t="n">
         <v>80.825</v>
       </c>
-      <c r="I59" t="n">
+      <c r="K59" t="n">
         <v>58.10850000000001</v>
       </c>
-      <c r="J59" t="n">
+      <c r="L59" t="n">
         <v>71.80000000000001</v>
       </c>
-      <c r="K59" t="n">
+      <c r="M59" t="n">
         <v>61.765</v>
       </c>
-      <c r="L59" t="n">
+      <c r="N59" t="n">
         <v>77.34999999999999</v>
       </c>
-      <c r="M59" t="n">
+      <c r="O59" t="n">
         <v>78.6352</v>
       </c>
-      <c r="N59" t="n">
+      <c r="P59" t="n">
         <v>71.81381034482757</v>
       </c>
     </row>
@@ -3529,30 +3887,36 @@
         </is>
       </c>
       <c r="F60" t="n">
+        <v>2.488341</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-76.40647</v>
+      </c>
+      <c r="H60" t="n">
         <v>67.97534</v>
       </c>
-      <c r="G60" t="n">
+      <c r="I60" t="n">
         <v>57.46</v>
       </c>
-      <c r="H60" t="n">
+      <c r="J60" t="n">
         <v>85.56925</v>
       </c>
-      <c r="I60" t="n">
+      <c r="K60" t="n">
         <v>95.02488000000001</v>
       </c>
-      <c r="J60" t="n">
+      <c r="L60" t="n">
         <v>74.40000000000001</v>
       </c>
-      <c r="K60" t="n">
+      <c r="M60" t="n">
         <v>46.97</v>
       </c>
-      <c r="L60" t="n">
+      <c r="N60" t="n">
         <v>60.81</v>
       </c>
-      <c r="M60" t="n">
+      <c r="O60" t="n">
         <v>91.29679999999999</v>
       </c>
-      <c r="N60" t="n">
+      <c r="P60" t="n">
         <v>72.43828375000001</v>
       </c>
     </row>
@@ -3581,30 +3945,36 @@
         </is>
       </c>
       <c r="F61" t="n">
+        <v>2.562222</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-76.503333</v>
+      </c>
+      <c r="H61" t="n">
         <v>72.50198827586208</v>
       </c>
-      <c r="G61" t="n">
+      <c r="I61" t="n">
         <v>80.5</v>
       </c>
-      <c r="H61" t="n">
+      <c r="J61" t="n">
         <v>78.78274999999999</v>
       </c>
-      <c r="I61" t="n">
+      <c r="K61" t="n">
         <v>87.74550000000001</v>
       </c>
-      <c r="J61" t="n">
+      <c r="L61" t="n">
         <v>56.5</v>
       </c>
-      <c r="K61" t="n">
+      <c r="M61" t="n">
         <v>44.935</v>
       </c>
-      <c r="L61" t="n">
+      <c r="N61" t="n">
         <v>67.95999999999999</v>
       </c>
-      <c r="M61" t="n">
+      <c r="O61" t="n">
         <v>91.2968</v>
       </c>
-      <c r="N61" t="n">
+      <c r="P61" t="n">
         <v>72.52775478448275</v>
       </c>
     </row>
@@ -3633,30 +4003,36 @@
         </is>
       </c>
       <c r="F62" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-76.42</v>
+      </c>
+      <c r="H62" t="n">
         <v>67.7861</v>
       </c>
-      <c r="G62" t="n">
+      <c r="I62" t="n">
         <v>50</v>
       </c>
-      <c r="H62" t="n">
+      <c r="J62" t="n">
         <v>87.23024999999998</v>
       </c>
-      <c r="I62" t="n">
+      <c r="K62" t="n">
         <v>96.52005</v>
       </c>
-      <c r="J62" t="n">
+      <c r="L62" t="n">
         <v>59.27800000000001</v>
       </c>
-      <c r="K62" t="n">
+      <c r="M62" t="n">
         <v>53.845</v>
       </c>
-      <c r="L62" t="n">
+      <c r="N62" t="n">
         <v>72.87</v>
       </c>
-      <c r="M62" t="n">
+      <c r="O62" t="n">
         <v>95.6284</v>
       </c>
-      <c r="N62" t="n">
+      <c r="P62" t="n">
         <v>72.89472499999999</v>
       </c>
     </row>
@@ -3685,30 +4061,36 @@
         </is>
       </c>
       <c r="F63" t="n">
+        <v>4.6115</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-74.08320000000001</v>
+      </c>
+      <c r="H63" t="n">
         <v>68.50991724137931</v>
       </c>
-      <c r="G63" t="n">
+      <c r="I63" t="n">
         <v>80.5</v>
       </c>
-      <c r="H63" t="n">
+      <c r="J63" t="n">
         <v>70.325</v>
       </c>
-      <c r="I63" t="n">
+      <c r="K63" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="J63" t="n">
+      <c r="L63" t="n">
         <v>59.59999999999999</v>
       </c>
-      <c r="K63" t="n">
+      <c r="M63" t="n">
         <v>54.56</v>
       </c>
-      <c r="L63" t="n">
+      <c r="N63" t="n">
         <v>78.23</v>
       </c>
-      <c r="M63" t="n">
+      <c r="O63" t="n">
         <v>91.46339999999999</v>
       </c>
-      <c r="N63" t="n">
+      <c r="P63" t="n">
         <v>75.38603965517243</v>
       </c>
     </row>

</xml_diff>